<commit_message>
Add two Family Room electrical items (interior dimmers, exterior switch)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="92">
   <si>
     <t xml:space="preserve">Location</t>
   </si>
@@ -73,6 +73,15 @@
   </si>
   <si>
     <t xml:space="preserve">Family Room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Put all interior lights on dimmers - the light in front of the bathroom is currently not on a dimmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change exterior light from dimmer to standard on/off switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Currently on a dimmer</t>
   </si>
   <si>
     <t xml:space="preserve">Painting</t>
@@ -298,10 +307,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
-    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0"/>
+    <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -419,7 +429,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -448,6 +458,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -464,7 +482,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -753,7 +771,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:J502"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -835,50 +853,52 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="7"/>
+      <c r="E4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4" t="s">
+      <c r="D5" s="7"/>
+      <c r="E5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="F5" s="7"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="s">
@@ -886,19 +906,17 @@
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="6"/>
-      <c r="H6" s="5" t="s">
-        <v>22</v>
-      </c>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
@@ -910,13 +928,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
@@ -924,17 +942,19 @@
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
@@ -942,19 +962,17 @@
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="6"/>
-      <c r="H9" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
@@ -966,13 +984,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
@@ -981,18 +999,18 @@
       <c r="F11" s="4"/>
       <c r="G11" s="6"/>
       <c r="H11" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
@@ -1000,19 +1018,17 @@
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="6"/>
-      <c r="H12" s="5" t="s">
-        <v>37</v>
-      </c>
+      <c r="H12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
@@ -1020,17 +1036,19 @@
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>38</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
@@ -1038,17 +1056,19 @@
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="6"/>
-      <c r="H14" s="5"/>
+      <c r="H14" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
@@ -1060,7 +1080,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>10</v>
@@ -1074,19 +1094,17 @@
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
@@ -1094,19 +1112,17 @@
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="H17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
@@ -1114,11 +1130,13 @@
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="6"/>
-      <c r="H18" s="5"/>
+      <c r="H18" s="5" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>10</v>
@@ -1132,17 +1150,19 @@
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="6"/>
-      <c r="H19" s="5"/>
+      <c r="H19" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
@@ -1154,13 +1174,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
@@ -1172,10 +1192,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>56</v>
@@ -1190,10 +1210,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>57</v>
@@ -1208,13 +1228,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
@@ -1226,10 +1246,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>60</v>
@@ -1243,21 +1263,37 @@
       <c r="H25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="5"/>
+      <c r="A26" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="E26" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="6"/>
       <c r="H26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="5"/>
+      <c r="A27" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F27" s="4"/>
       <c r="G27" s="6"/>
       <c r="H27" s="5"/>
@@ -5991,6 +6027,26 @@
       <c r="F500" s="4"/>
       <c r="G500" s="6"/>
       <c r="H500" s="5"/>
+    </row>
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A501" s="4"/>
+      <c r="B501" s="4"/>
+      <c r="C501" s="5"/>
+      <c r="D501" s="4"/>
+      <c r="E501" s="4"/>
+      <c r="F501" s="4"/>
+      <c r="G501" s="6"/>
+      <c r="H501" s="5"/>
+    </row>
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A502" s="4"/>
+      <c r="B502" s="4"/>
+      <c r="C502" s="5"/>
+      <c r="D502" s="4"/>
+      <c r="E502" s="4"/>
+      <c r="F502" s="4"/>
+      <c r="G502" s="6"/>
+      <c r="H502" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H500"/>
@@ -6035,186 +6091,186 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>59</v>
-      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>45</v>
+      <c r="A17" s="11" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>48</v>
+      <c r="A18" s="11" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>50</v>
+      <c r="A19" s="11" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
-        <v>51</v>
+      <c r="A20" s="11" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>55</v>
+      <c r="A21" s="11" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -6241,60 +6297,60 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>86</v>
+      <c r="A1" s="12" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="11" t="n">
+      <c r="A3" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="13" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Not Started")</f>
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="11" t="n">
+      <c r="A5" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="11" t="n">
+      <c r="A7" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" s="12" t="n">
+      <c r="A8" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="14" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add Downstairs Bathroom items (sheetrock fill, pencil line cleanup)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
   <si>
     <t xml:space="preserve">Location</t>
   </si>
@@ -117,6 +117,18 @@
     <t xml:space="preserve">Set up powder room (general)</t>
   </si>
   <si>
+    <t xml:space="preserve">Downstairs Bathroom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drywall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill in sheetrock in the area under the medicine cabinet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean up pencil lines above the medicine cabinet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hallway</t>
   </si>
   <si>
@@ -265,9 +277,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dining</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drywall</t>
   </si>
   <si>
     <t xml:space="preserve">Bath 1</t>
@@ -429,7 +438,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -475,6 +484,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -771,7 +784,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J502"/>
+  <dimension ref="A1:J504"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -853,39 +866,39 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="8"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="6"/>
       <c r="H4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="6"/>
       <c r="H5" s="5" t="s">
         <v>18</v>
       </c>
@@ -983,41 +996,39 @@
       <c r="H10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>10</v>
+      <c r="B11" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="5" t="s">
-        <v>32</v>
-      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4" t="s">
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="6"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
       <c r="H12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1025,10 +1036,10 @@
         <v>34</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
@@ -1037,18 +1048,18 @@
       <c r="F13" s="4"/>
       <c r="G13" s="6"/>
       <c r="H13" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
@@ -1056,19 +1067,17 @@
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="6"/>
-      <c r="H14" s="5" t="s">
-        <v>40</v>
-      </c>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
@@ -1076,14 +1085,16 @@
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="5"/>
+      <c r="H15" s="5" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>43</v>
@@ -1094,17 +1105,19 @@
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="5"/>
+      <c r="H16" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
@@ -1122,7 +1135,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
@@ -1130,19 +1143,17 @@
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="6"/>
-      <c r="H18" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
@@ -1150,19 +1161,17 @@
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="6"/>
-      <c r="H19" s="5" t="s">
-        <v>50</v>
-      </c>
+      <c r="H19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
@@ -1170,17 +1179,19 @@
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="6"/>
-      <c r="H20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
@@ -1188,14 +1199,16 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="6"/>
-      <c r="H21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>56</v>
@@ -1210,13 +1223,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
@@ -1231,10 +1244,10 @@
         <v>58</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
@@ -1249,10 +1262,10 @@
         <v>58</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
@@ -1264,13 +1277,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
@@ -1282,13 +1295,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
@@ -1299,21 +1312,37 @@
       <c r="H27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="5"/>
+      <c r="A28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="E28" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F28" s="4"/>
       <c r="G28" s="6"/>
       <c r="H28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="5"/>
+      <c r="A29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>67</v>
+      </c>
       <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="6"/>
       <c r="H29" s="5"/>
@@ -6028,7 +6057,7 @@
       <c r="G500" s="6"/>
       <c r="H500" s="5"/>
     </row>
-    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A501" s="4"/>
       <c r="B501" s="4"/>
       <c r="C501" s="5"/>
@@ -6038,7 +6067,7 @@
       <c r="G501" s="6"/>
       <c r="H501" s="5"/>
     </row>
-    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A502" s="4"/>
       <c r="B502" s="4"/>
       <c r="C502" s="5"/>
@@ -6047,6 +6076,26 @@
       <c r="F502" s="4"/>
       <c r="G502" s="6"/>
       <c r="H502" s="5"/>
+    </row>
+    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A503" s="4"/>
+      <c r="B503" s="4"/>
+      <c r="C503" s="5"/>
+      <c r="D503" s="4"/>
+      <c r="E503" s="4"/>
+      <c r="F503" s="4"/>
+      <c r="G503" s="6"/>
+      <c r="H503" s="5"/>
+    </row>
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A504" s="4"/>
+      <c r="B504" s="4"/>
+      <c r="C504" s="5"/>
+      <c r="D504" s="4"/>
+      <c r="E504" s="4"/>
+      <c r="F504" s="4"/>
+      <c r="G504" s="6"/>
+      <c r="H504" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H500"/>
@@ -6084,7 +6133,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="1" width="22"/>
@@ -6092,24 +6141,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>28</v>
@@ -6118,35 +6167,35 @@
         <v>12</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6154,18 +6203,18 @@
         <v>15</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6173,12 +6222,12 @@
         <v>9</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>80</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>19</v>
@@ -6186,10 +6235,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6197,12 +6246,12 @@
         <v>27</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>21</v>
@@ -6210,10 +6259,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6221,56 +6270,61 @@
         <v>23</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>58</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -6297,60 +6351,60 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>89</v>
+      <c r="A1" s="13" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="13" t="n">
+        <v>93</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="14" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Not Started")</f>
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="13" t="n">
+        <v>76</v>
+      </c>
+      <c r="B5" s="14" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="B6" s="14" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B7" s="13" t="n">
+        <v>82</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B8" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add protective film removal item for downstairs bathroom medicine cabinet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="96">
   <si>
     <t xml:space="preserve">Location</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fill in sheetrock in the area under the medicine cabinet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove protective film from the medicine cabinet - still on, making the mirror look dark</t>
   </si>
   <si>
     <t xml:space="preserve">Clean up pencil lines above the medicine cabinet</t>
@@ -438,7 +441,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -484,10 +487,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -784,7 +783,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J504"/>
+  <dimension ref="A1:J505"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -996,21 +995,21 @@
       <c r="H10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7" t="s">
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1018,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>33</v>
@@ -1033,13 +1032,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
@@ -1047,19 +1046,17 @@
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="5" t="s">
-        <v>36</v>
-      </c>
+      <c r="H13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
@@ -1067,17 +1064,19 @@
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="6"/>
-      <c r="H14" s="5"/>
+      <c r="H14" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
@@ -1085,19 +1084,17 @@
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="H15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
@@ -1106,18 +1103,18 @@
       <c r="F16" s="4"/>
       <c r="G16" s="6"/>
       <c r="H16" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
@@ -1125,11 +1122,13 @@
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="5"/>
+      <c r="H17" s="5" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>10</v>
@@ -1147,10 +1146,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>48</v>
@@ -1165,13 +1164,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
@@ -1179,19 +1178,17 @@
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="6"/>
-      <c r="H20" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="H20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
@@ -1200,18 +1197,18 @@
       <c r="F21" s="4"/>
       <c r="G21" s="6"/>
       <c r="H21" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
@@ -1219,17 +1216,19 @@
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="6"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
@@ -1244,10 +1243,10 @@
         <v>58</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
@@ -1259,10 +1258,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>61</v>
@@ -1277,13 +1276,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
@@ -1295,10 +1294,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>64</v>
@@ -1313,10 +1312,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>65</v>
@@ -1331,13 +1330,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
@@ -1348,11 +1347,19 @@
       <c r="H29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="5"/>
+      <c r="A30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="E30" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="6"/>
       <c r="H30" s="5"/>
@@ -6077,7 +6084,7 @@
       <c r="G502" s="6"/>
       <c r="H502" s="5"/>
     </row>
-    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A503" s="4"/>
       <c r="B503" s="4"/>
       <c r="C503" s="5"/>
@@ -6087,7 +6094,7 @@
       <c r="G503" s="6"/>
       <c r="H503" s="5"/>
     </row>
-    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A504" s="4"/>
       <c r="B504" s="4"/>
       <c r="C504" s="5"/>
@@ -6096,6 +6103,16 @@
       <c r="F504" s="4"/>
       <c r="G504" s="6"/>
       <c r="H504" s="5"/>
+    </row>
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A505" s="4"/>
+      <c r="B505" s="4"/>
+      <c r="C505" s="5"/>
+      <c r="D505" s="4"/>
+      <c r="E505" s="4"/>
+      <c r="F505" s="4"/>
+      <c r="G505" s="6"/>
+      <c r="H505" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H500"/>
@@ -6141,24 +6158,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>28</v>
@@ -6167,35 +6184,35 @@
         <v>12</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6203,18 +6220,18 @@
         <v>15</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6227,7 +6244,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>19</v>
@@ -6235,10 +6252,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6246,12 +6263,12 @@
         <v>27</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>21</v>
@@ -6259,10 +6276,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6270,60 +6287,60 @@
         <v>23</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>30</v>
       </c>
     </row>
@@ -6351,60 +6368,60 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
-        <v>92</v>
+      <c r="A1" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="B3" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="B3" s="13" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Not Started")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>77</v>
+      </c>
+      <c r="B5" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="14" t="n">
+        <v>81</v>
+      </c>
+      <c r="B6" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="15" t="n">
+        <v>95</v>
+      </c>
+      <c r="B8" s="14" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add upstairs bathroom bulb swap to 4000K cool white
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="98">
   <si>
     <t xml:space="preserve">Location</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t xml:space="preserve">Change timer switch to an occupancy sensor switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace 2700K vanity bulb with 4000K (cool white) - current warm color not liked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current bulb: 450 lumens LED, ~40W equivalent, E26 base. Buy 4000K replacement</t>
   </si>
   <si>
     <t xml:space="preserve">Install medicine cabinet</t>
@@ -783,7 +789,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J505"/>
+  <dimension ref="A1:J506"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -1013,21 +1019,21 @@
       <c r="H11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7" t="s">
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1163,29 +1169,31 @@
       <c r="H19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>28</v>
+      <c r="B20" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4" t="s">
+      <c r="D20" s="7"/>
+      <c r="E20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="5"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>51</v>
@@ -1196,19 +1204,17 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="6"/>
-      <c r="H21" s="5" t="s">
-        <v>52</v>
-      </c>
+      <c r="H21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
@@ -1217,18 +1223,18 @@
       <c r="F22" s="4"/>
       <c r="G22" s="6"/>
       <c r="H22" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
@@ -1236,7 +1242,9 @@
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="6"/>
-      <c r="H23" s="5"/>
+      <c r="H23" s="5" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
@@ -1246,7 +1254,7 @@
         <v>10</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
@@ -1258,13 +1266,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
@@ -1276,13 +1284,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
@@ -1294,10 +1302,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>64</v>
@@ -1312,13 +1320,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
@@ -1330,13 +1338,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
@@ -1348,10 +1356,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>68</v>
@@ -1365,11 +1373,19 @@
       <c r="H30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="5"/>
+      <c r="A31" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="6"/>
       <c r="H31" s="5"/>
@@ -6104,7 +6120,7 @@
       <c r="G504" s="6"/>
       <c r="H504" s="5"/>
     </row>
-    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A505" s="4"/>
       <c r="B505" s="4"/>
       <c r="C505" s="5"/>
@@ -6113,6 +6129,16 @@
       <c r="F505" s="4"/>
       <c r="G505" s="6"/>
       <c r="H505" s="5"/>
+    </row>
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A506" s="4"/>
+      <c r="B506" s="4"/>
+      <c r="C506" s="5"/>
+      <c r="D506" s="4"/>
+      <c r="E506" s="4"/>
+      <c r="F506" s="4"/>
+      <c r="G506" s="6"/>
+      <c r="H506" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H500"/>
@@ -6158,24 +6184,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>28</v>
@@ -6184,35 +6210,35 @@
         <v>12</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6220,15 +6246,15 @@
         <v>15</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>40</v>
@@ -6252,10 +6278,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6263,7 +6289,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6276,10 +6302,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6287,7 +6313,7 @@
         <v>23</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6295,7 +6321,7 @@
         <v>43</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6303,40 +6329,40 @@
         <v>46</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6369,16 +6395,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6387,12 +6413,12 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Not Started")</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
@@ -6401,7 +6427,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
@@ -6410,7 +6436,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
@@ -6419,7 +6445,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>

</xml_diff>

<commit_message>
Bump upstairs bathroom replacement bulb to 60W equivalent
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -174,10 +174,10 @@
     <t xml:space="preserve">Change timer switch to an occupancy sensor switch</t>
   </si>
   <si>
-    <t xml:space="preserve">Replace 2700K vanity bulb with 4000K (cool white) - current warm color not liked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current bulb: 450 lumens LED, ~40W equivalent, E26 base. Buy 4000K replacement</t>
+    <t xml:space="preserve">Replace 2700K vanity bulb with 4000K (cool white), 60W equivalent - current warm color not liked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy: 4000K, ~800 lumens (60W equivalent), E26 base. Current bulb is only 450 lm (~40W equiv)</t>
   </si>
   <si>
     <t xml:space="preserve">Install medicine cabinet</t>
@@ -325,11 +325,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0"/>
-    <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -447,7 +446,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -476,14 +475,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -500,7 +491,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1169,21 +1160,21 @@
       <c r="H19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7" t="s">
+      <c r="D20" s="4"/>
+      <c r="E20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="8"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="6"/>
       <c r="H20" s="5" t="s">
         <v>50</v>
       </c>
@@ -6130,7 +6121,7 @@
       <c r="G505" s="6"/>
       <c r="H505" s="5"/>
     </row>
-    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A506" s="4"/>
       <c r="B506" s="4"/>
       <c r="C506" s="5"/>
@@ -6183,190 +6174,190 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="8" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="9" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="9" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="9" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="9" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="9" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="9" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="9" t="s">
         <v>30</v>
       </c>
     </row>
@@ -6394,60 +6385,60 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="11" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Not Started")</f>
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="12" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Apply clarifications from earlier walkthrough draft
Dehumidifier set to 45%, HVAC thermostat error to clear, medicine
cabinet Monday arrival, both upstairs bath switches on occupancy
sensors (60-minute timer removed).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ApWXef9kmSdQmFnJQR1CYZ
</commit_message>
<xml_diff>
--- a/461-anderson-punch-list.xlsx
+++ b/461-anderson-punch-list.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="99">
   <si>
     <t xml:space="preserve">Location</t>
   </si>
@@ -171,7 +171,7 @@
     <t xml:space="preserve">Fix vanity light - flickers when turned on</t>
   </si>
   <si>
-    <t xml:space="preserve">Change timer switch to an occupancy sensor switch</t>
+    <t xml:space="preserve">Put both light switches on occupancy sensors - remove the switch with the 60-minute timer</t>
   </si>
   <si>
     <t xml:space="preserve">Replace 2700K vanity bulb with 4000K (cool white), 60W equivalent - current warm color not liked</t>
@@ -183,6 +183,9 @@
     <t xml:space="preserve">Install medicine cabinet</t>
   </si>
   <si>
+    <t xml:space="preserve">Cabinet arriving Mon Jul 27</t>
+  </si>
+  <si>
     <t xml:space="preserve">Concierge Bathroom</t>
   </si>
   <si>
@@ -216,10 +219,10 @@
     <t xml:space="preserve">HVAC</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm HVAC is working</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm whole-home dehumidifier is working</t>
+    <t xml:space="preserve">Confirm HVAC is working - clear the error still showing on the HVAC/thermostat screen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turn on whole-home dehumidifier, set to 45%, and confirm working</t>
   </si>
   <si>
     <t xml:space="preserve">Garage</t>
@@ -1195,17 +1198,19 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="6"/>
-      <c r="H21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
@@ -1214,18 +1219,18 @@
       <c r="F22" s="4"/>
       <c r="G22" s="6"/>
       <c r="H22" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
@@ -1234,18 +1239,18 @@
       <c r="F23" s="4"/>
       <c r="G23" s="6"/>
       <c r="H23" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
@@ -1257,13 +1262,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
@@ -1275,13 +1280,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
@@ -1293,13 +1298,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
@@ -1311,13 +1316,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
@@ -1329,13 +1334,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
@@ -1347,13 +1352,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
@@ -1365,13 +1370,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
@@ -6175,24 +6180,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>28</v>
@@ -6201,35 +6206,35 @@
         <v>12</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6237,15 +6242,15 @@
         <v>15</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>40</v>
@@ -6269,10 +6274,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6280,7 +6285,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6293,10 +6298,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6304,7 +6309,7 @@
         <v>23</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6312,7 +6317,7 @@
         <v>43</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6320,40 +6325,40 @@
         <v>46</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6386,12 +6391,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B3" s="11" t="n">
         <f aca="false">COUNTA('Punch List'!C2:C500)</f>
@@ -6409,7 +6414,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"In Progress")</f>
@@ -6418,7 +6423,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Blocked")</f>
@@ -6427,7 +6432,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF('Punch List'!E2:E500,"Done")</f>
@@ -6436,7 +6441,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM('Punch List'!G2:G500)</f>

</xml_diff>